<commit_message>
Worked on New Part Request API and Part Details Import Issue Fixed
</commit_message>
<xml_diff>
--- a/OraRegaAV/FormatFiles/PartDetailsFormatFile.xlsx
+++ b/OraRegaAV/FormatFiles/PartDetailsFormatFile.xlsx
@@ -569,9 +569,12 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q1:Q1048576">
       <formula1>"Active,In Active"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L1048576">
+      <formula1>"Good,DOA,Defective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>